<commit_message>
Polish: Projects tab always opens project list, global home without context bar, accurate copy, shared popup footer
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/poc-output/m9-chromium/export-filtered.xlsx
+++ b/poc-output/m9-chromium/export-filtered.xlsx
@@ -293,7 +293,7 @@
         <v>46315.41677083333</v>
       </c>
       <c r="P2" s="3">
-        <v>46317.51144824074</v>
+        <v>46317.53180380787</v>
       </c>
       <c r="Q2" s="8">
         <v>0</v>
@@ -365,7 +365,7 @@
         <v>46315.417245370365</v>
       </c>
       <c r="P3" s="3">
-        <v>46317.5114486574</v>
+        <v>46317.53180420139</v>
       </c>
       <c r="Q3" s="8">
         <v>0</v>
@@ -437,7 +437,7 @@
         <v>46315.417025462964</v>
       </c>
       <c r="P4" s="3">
-        <v>46317.51154056713</v>
+        <v>46317.53189219907</v>
       </c>
       <c r="Q4" s="8">
         <v>0</v>
@@ -509,7 +509,7 @@
         <v>46315.41680555556</v>
       </c>
       <c r="P5" s="3">
-        <v>46317.5114486574</v>
+        <v>46317.53180420139</v>
       </c>
       <c r="Q5" s="8">
         <v>1</v>
@@ -581,7 +581,7 @@
         <v>46315.41728009259</v>
       </c>
       <c r="P6" s="3">
-        <v>46317.51152513889</v>
+        <v>46317.531876574074</v>
       </c>
       <c r="Q6" s="8">
         <v>0</v>
@@ -653,7 +653,7 @@
         <v>46315.41706018518</v>
       </c>
       <c r="P7" s="3">
-        <v>46317.51144902778</v>
+        <v>46317.531804583334</v>
       </c>
       <c r="Q7" s="8">
         <v>0</v>
@@ -720,7 +720,7 @@
         <v>46315.41684027778</v>
       </c>
       <c r="P8" s="3">
-        <v>46317.51144824074</v>
+        <v>46317.53180380787</v>
       </c>
       <c r="Q8" s="8">
         <v>3</v>
@@ -792,7 +792,7 @@
         <v>46315.41731481481</v>
       </c>
       <c r="P9" s="3">
-        <v>46317.51152513889</v>
+        <v>46317.531876574074</v>
       </c>
       <c r="Q9" s="8">
         <v>0</v>
@@ -864,7 +864,7 @@
         <v>46315.4170949074</v>
       </c>
       <c r="P10" s="3">
-        <v>46317.5114486574</v>
+        <v>46317.53180420139</v>
       </c>
       <c r="Q10" s="8">
         <v>0</v>
@@ -936,7 +936,7 @@
         <v>46315.416874999995</v>
       </c>
       <c r="P11" s="3">
-        <v>46317.5114486574</v>
+        <v>46317.53180420139</v>
       </c>
       <c r="Q11" s="8">
         <v>1</v>
@@ -1008,7 +1008,7 @@
         <v>46315.417349537034</v>
       </c>
       <c r="P12" s="3">
-        <v>46317.51144902778</v>
+        <v>46317.531804583334</v>
       </c>
       <c r="Q12" s="8">
         <v>0</v>
@@ -1080,7 +1080,7 @@
         <v>46315.417129629626</v>
       </c>
       <c r="P13" s="3">
-        <v>46317.51144902778</v>
+        <v>46317.531804583334</v>
       </c>
       <c r="Q13" s="8">
         <v>0</v>
@@ -1157,7 +1157,7 @@
         <v>46315.41690972222</v>
       </c>
       <c r="P14" s="3">
-        <v>46317.51144824074</v>
+        <v>46317.53180380787</v>
       </c>
       <c r="Q14" s="8">
         <v>0</v>
@@ -1234,7 +1234,7 @@
         <v>46315.41668981481</v>
       </c>
       <c r="P15" s="3">
-        <v>46317.5114486574</v>
+        <v>46317.53180420139</v>
       </c>
       <c r="Q15" s="8">
         <v>0</v>
@@ -1306,7 +1306,7 @@
         <v>46315.41716435185</v>
       </c>
       <c r="P16" s="3">
-        <v>46317.5114486574</v>
+        <v>46317.53180420139</v>
       </c>
       <c r="Q16" s="8">
         <v>0</v>
@@ -1383,7 +1383,7 @@
         <v>46315.41694444444</v>
       </c>
       <c r="P17" s="3">
-        <v>46317.51144902778</v>
+        <v>46317.531804583334</v>
       </c>
       <c r="Q17" s="8">
         <v>1</v>
@@ -1460,7 +1460,7 @@
         <v>46315.41672453703</v>
       </c>
       <c r="P18" s="3">
-        <v>46317.51144902778</v>
+        <v>46317.531804583334</v>
       </c>
       <c r="Q18" s="8">
         <v>0</v>
@@ -1537,7 +1537,7 @@
         <v>46315.41719907407</v>
       </c>
       <c r="P19" s="3">
-        <v>46317.51154056713</v>
+        <v>46317.53189219907</v>
       </c>
       <c r="Q19" s="8">
         <v>0</v>
@@ -1614,7 +1614,7 @@
         <v>46315.416979166665</v>
       </c>
       <c r="P20" s="3">
-        <v>46317.51144824074</v>
+        <v>46317.53180380787</v>
       </c>
       <c r="Q20" s="8">
         <v>0</v>
@@ -1691,7 +1691,7 @@
         <v>46315.41675925926</v>
       </c>
       <c r="P21" s="3">
-        <v>46317.5114486574</v>
+        <v>46317.53180420139</v>
       </c>
       <c r="Q21" s="8">
         <v>0</v>
@@ -1768,7 +1768,7 @@
         <v>46315.417233796295</v>
       </c>
       <c r="P22" s="3">
-        <v>46317.51154056713</v>
+        <v>46317.53189219907</v>
       </c>
       <c r="Q22" s="8">
         <v>0</v>
@@ -1845,7 +1845,7 @@
         <v>46315.41701388889</v>
       </c>
       <c r="P23" s="3">
-        <v>46317.51144902778</v>
+        <v>46317.531804583334</v>
       </c>
       <c r="Q23" s="8">
         <v>3</v>
@@ -1917,7 +1917,7 @@
         <v>46315.41679398148</v>
       </c>
       <c r="P24" s="3">
-        <v>46317.51152513889</v>
+        <v>46317.531876574074</v>
       </c>
       <c r="Q24" s="8">
         <v>0</v>
@@ -1994,7 +1994,7 @@
         <v>46315.41726851852</v>
       </c>
       <c r="P25" s="3">
-        <v>46317.51144902778</v>
+        <v>46317.531804583334</v>
       </c>
       <c r="Q25" s="8">
         <v>0</v>
@@ -2071,7 +2071,7 @@
         <v>46315.41726851852</v>
       </c>
       <c r="P26" s="3">
-        <v>46317.51154056713</v>
+        <v>46317.53189219907</v>
       </c>
       <c r="Q26" s="8">
         <v>0</v>
@@ -2148,7 +2148,7 @@
         <v>46315.41704861111</v>
       </c>
       <c r="P27" s="3">
-        <v>46317.51144824074</v>
+        <v>46317.53180380787</v>
       </c>
       <c r="Q27" s="8">
         <v>0</v>
@@ -2225,7 +2225,7 @@
         <v>46315.4168287037</v>
       </c>
       <c r="P28" s="3">
-        <v>46317.51152513889</v>
+        <v>46317.531876574074</v>
       </c>
       <c r="Q28" s="8">
         <v>0</v>
@@ -2302,7 +2302,7 @@
         <v>46315.41730324074</v>
       </c>
       <c r="P29" s="3">
-        <v>46317.5114486574</v>
+        <v>46317.53180420139</v>
       </c>
       <c r="Q29" s="8">
         <v>0</v>
@@ -2379,7 +2379,7 @@
         <v>46315.417083333334</v>
       </c>
       <c r="P30" s="3">
-        <v>46317.51144902778</v>
+        <v>46317.531804583334</v>
       </c>
       <c r="Q30" s="8">
         <v>1</v>
@@ -2456,7 +2456,7 @@
         <v>46315.416863425926</v>
       </c>
       <c r="P31" s="3">
-        <v>46317.51144902778</v>
+        <v>46317.531804583334</v>
       </c>
       <c r="Q31" s="8">
         <v>0</v>
@@ -2533,7 +2533,7 @@
         <v>46315.417337962965</v>
       </c>
       <c r="P32" s="3">
-        <v>46317.51144902778</v>
+        <v>46317.531804583334</v>
       </c>
       <c r="Q32" s="8">
         <v>0</v>
@@ -2610,7 +2610,7 @@
         <v>46315.417337962965</v>
       </c>
       <c r="P33" s="3">
-        <v>46317.51144824074</v>
+        <v>46317.53180380787</v>
       </c>
       <c r="Q33" s="8">
         <v>0</v>
@@ -2682,7 +2682,7 @@
         <v>46315.41711805556</v>
       </c>
       <c r="P34" s="3">
-        <v>46317.51144824074</v>
+        <v>46317.53180380787</v>
       </c>
       <c r="Q34" s="8">
         <v>0</v>
@@ -2759,7 +2759,7 @@
         <v>46315.41689814815</v>
       </c>
       <c r="P35" s="3">
-        <v>46317.5114486574</v>
+        <v>46317.53180420139</v>
       </c>
       <c r="Q35" s="8">
         <v>0</v>
@@ -2836,7 +2836,7 @@
         <v>46315.41667824074</v>
       </c>
       <c r="P36" s="3">
-        <v>46317.5114486574</v>
+        <v>46317.53180420139</v>
       </c>
       <c r="Q36" s="8">
         <v>0</v>
@@ -2913,7 +2913,7 @@
         <v>46315.41715277778</v>
       </c>
       <c r="P37" s="3">
-        <v>46317.51144902778</v>
+        <v>46317.531804583334</v>
       </c>
       <c r="Q37" s="8">
         <v>1</v>
@@ -2990,7 +2990,7 @@
         <v>46315.41693287037</v>
       </c>
       <c r="P38" s="3">
-        <v>46317.51144902778</v>
+        <v>46317.531804583334</v>
       </c>
       <c r="Q38" s="8">
         <v>0</v>
@@ -3067,7 +3067,7 @@
         <v>46315.416712962964</v>
       </c>
       <c r="P39" s="3">
-        <v>46317.51144824074</v>
+        <v>46317.53180380787</v>
       </c>
       <c r="Q39" s="8">
         <v>0</v>
@@ -3144,7 +3144,7 @@
         <v>46315.4171875</v>
       </c>
       <c r="P40" s="3">
-        <v>46317.5114486574</v>
+        <v>46317.53180420139</v>
       </c>
       <c r="Q40" s="8">
         <v>3</v>
@@ -3221,7 +3221,7 @@
         <v>46315.416967592595</v>
       </c>
       <c r="P41" s="3">
-        <v>46317.5114486574</v>
+        <v>46317.53180420139</v>
       </c>
       <c r="Q41" s="8">
         <v>0</v>
@@ -3293,7 +3293,7 @@
         <v>46315.41674768519</v>
       </c>
       <c r="P42" s="3">
-        <v>46317.51154056713</v>
+        <v>46317.53189219907</v>
       </c>
       <c r="Q42" s="8">
         <v>0</v>
@@ -3370,7 +3370,7 @@
         <v>46315.417222222226</v>
       </c>
       <c r="P43" s="3">
-        <v>46317.51144902778</v>
+        <v>46317.531804583334</v>
       </c>
       <c r="Q43" s="8">
         <v>1</v>
@@ -3447,7 +3447,7 @@
         <v>46315.41700231482</v>
       </c>
       <c r="P44" s="3">
-        <v>46317.51144902778</v>
+        <v>46317.531804583334</v>
       </c>
       <c r="Q44" s="8">
         <v>0</v>
@@ -3524,7 +3524,7 @@
         <v>46315.41678240741</v>
       </c>
       <c r="P45" s="3">
-        <v>46317.51154056713</v>
+        <v>46317.53189219907</v>
       </c>
       <c r="Q45" s="8">
         <v>0</v>
@@ -3601,7 +3601,7 @@
         <v>46315.41725694445</v>
       </c>
       <c r="P46" s="3">
-        <v>46317.5114486574</v>
+        <v>46317.53180420139</v>
       </c>
       <c r="Q46" s="8">
         <v>0</v>
@@ -3678,7 +3678,7 @@
         <v>46315.41703703704</v>
       </c>
       <c r="P47" s="3">
-        <v>46317.5114486574</v>
+        <v>46317.53180420139</v>
       </c>
       <c r="Q47" s="8">
         <v>0</v>
@@ -3755,7 +3755,7 @@
         <v>46315.41681712963</v>
       </c>
       <c r="P48" s="3">
-        <v>46317.5114486574</v>
+        <v>46317.53180420139</v>
       </c>
       <c r="Q48" s="8">
         <v>0</v>
@@ -3832,7 +3832,7 @@
         <v>46315.41729166667</v>
       </c>
       <c r="P49" s="3">
-        <v>46317.51144902778</v>
+        <v>46317.531804583334</v>
       </c>
       <c r="Q49" s="8">
         <v>1</v>
@@ -3904,7 +3904,7 @@
         <v>46315.417071759264</v>
       </c>
       <c r="P50" s="3">
-        <v>46317.51144902778</v>
+        <v>46317.531804583334</v>
       </c>
       <c r="Q50" s="8">
         <v>0</v>
@@ -3981,7 +3981,7 @@
         <v>46315.416851851856</v>
       </c>
       <c r="P51" s="3">
-        <v>46317.51144824074</v>
+        <v>46317.53180380787</v>
       </c>
       <c r="Q51" s="8">
         <v>0</v>
@@ -4058,7 +4058,7 @@
         <v>46315.41732638889</v>
       </c>
       <c r="P52" s="3">
-        <v>46317.5114486574</v>
+        <v>46317.53180420139</v>
       </c>
       <c r="Q52" s="8">
         <v>0</v>
@@ -4135,7 +4135,7 @@
         <v>46315.41710648148</v>
       </c>
       <c r="P53" s="3">
-        <v>46317.5114486574</v>
+        <v>46317.53180420139</v>
       </c>
       <c r="Q53" s="8">
         <v>0</v>
@@ -4212,7 +4212,7 @@
         <v>46315.41688657408</v>
       </c>
       <c r="P54" s="3">
-        <v>46317.5114486574</v>
+        <v>46317.53180420139</v>
       </c>
       <c r="Q54" s="8">
         <v>0</v>
@@ -4289,7 +4289,7 @@
         <v>46315.41666666667</v>
       </c>
       <c r="P55" s="3">
-        <v>46317.51144902778</v>
+        <v>46317.531804583334</v>
       </c>
       <c r="Q55" s="8">
         <v>3</v>
@@ -4366,7 +4366,7 @@
         <v>46315.4171412037</v>
       </c>
       <c r="P56" s="3">
-        <v>46317.51144902778</v>
+        <v>46317.531804583334</v>
       </c>
       <c r="Q56" s="8">
         <v>0</v>
@@ -4443,7 +4443,7 @@
         <v>46315.416921296295</v>
       </c>
       <c r="P57" s="3">
-        <v>46317.51144824074</v>
+        <v>46317.53180380787</v>
       </c>
       <c r="Q57" s="8">
         <v>0</v>
@@ -4515,7 +4515,7 @@
         <v>46315.41670138889</v>
       </c>
       <c r="P58" s="3">
-        <v>46317.5114486574</v>
+        <v>46317.53180420139</v>
       </c>
       <c r="Q58" s="8">
         <v>0</v>
@@ -4592,7 +4592,7 @@
         <v>46315.417175925926</v>
       </c>
       <c r="P59" s="3">
-        <v>46317.5114486574</v>
+        <v>46317.53180420139</v>
       </c>
       <c r="Q59" s="8">
         <v>0</v>
@@ -4669,7 +4669,7 @@
         <v>46315.41695601852</v>
       </c>
       <c r="P60" s="3">
-        <v>46317.51154056713</v>
+        <v>46317.53189219907</v>
       </c>
       <c r="Q60" s="8">
         <v>0</v>
@@ -4746,7 +4746,7 @@
         <v>46315.41673611111</v>
       </c>
       <c r="P61" s="3">
-        <v>46317.51144902778</v>
+        <v>46317.531804583334</v>
       </c>
       <c r="Q61" s="8">
         <v>1</v>
@@ -4823,7 +4823,7 @@
         <v>46315.41721064815</v>
       </c>
       <c r="P62" s="3">
-        <v>46317.51152513889</v>
+        <v>46317.531876574074</v>
       </c>
       <c r="Q62" s="8">
         <v>0</v>
@@ -4900,7 +4900,7 @@
         <v>46315.41699074074</v>
       </c>
       <c r="P63" s="3">
-        <v>46317.51154056713</v>
+        <v>46317.53189219907</v>
       </c>
       <c r="Q63" s="8">
         <v>0</v>
@@ -4977,7 +4977,7 @@
         <v>46315.41677083333</v>
       </c>
       <c r="P64" s="3">
-        <v>46317.5114486574</v>
+        <v>46317.53180420139</v>
       </c>
       <c r="Q64" s="8">
         <v>0</v>
@@ -5054,7 +5054,7 @@
         <v>46315.417245370365</v>
       </c>
       <c r="P65" s="3">
-        <v>46317.51152513889</v>
+        <v>46317.531876574074</v>
       </c>
       <c r="Q65" s="8">
         <v>0</v>
@@ -5126,7 +5126,7 @@
         <v>46315.417025462964</v>
       </c>
       <c r="P66" s="3">
-        <v>46317.51144902778</v>
+        <v>46317.531804583334</v>
       </c>
       <c r="Q66" s="8">
         <v>0</v>
@@ -5203,7 +5203,7 @@
         <v>46315.41680555556</v>
       </c>
       <c r="P67" s="3">
-        <v>46317.51144902778</v>
+        <v>46317.531804583334</v>
       </c>
       <c r="Q67" s="8">
         <v>1</v>
@@ -5280,7 +5280,7 @@
         <v>46315.41728009259</v>
       </c>
       <c r="P68" s="3">
-        <v>46317.51144902778</v>
+        <v>46317.531804583334</v>
       </c>
       <c r="Q68" s="8">
         <v>0</v>
@@ -5357,7 +5357,7 @@
         <v>46315.41728009259</v>
       </c>
       <c r="P69" s="3">
-        <v>46317.51152513889</v>
+        <v>46317.531876574074</v>
       </c>
       <c r="Q69" s="8">
         <v>0</v>
@@ -5434,7 +5434,7 @@
         <v>46315.41706018518</v>
       </c>
       <c r="P70" s="3">
-        <v>46317.51144824074</v>
+        <v>46317.53180380787</v>
       </c>
       <c r="Q70" s="8">
         <v>0</v>
@@ -5511,7 +5511,7 @@
         <v>46315.41684027778</v>
       </c>
       <c r="P71" s="3">
-        <v>46317.5114486574</v>
+        <v>46317.53180420139</v>
       </c>
       <c r="Q71" s="8">
         <v>3</v>
@@ -5588,7 +5588,7 @@
         <v>46315.41731481481</v>
       </c>
       <c r="P72" s="3">
-        <v>46317.5114486574</v>
+        <v>46317.53180420139</v>
       </c>
       <c r="Q72" s="8">
         <v>0</v>
@@ -5665,7 +5665,7 @@
         <v>46315.4170949074</v>
       </c>
       <c r="P73" s="3">
-        <v>46317.51144902778</v>
+        <v>46317.531804583334</v>
       </c>
       <c r="Q73" s="8">
         <v>0</v>
@@ -5742,7 +5742,7 @@
         <v>46315.416874999995</v>
       </c>
       <c r="P74" s="3">
-        <v>46317.51144902778</v>
+        <v>46317.531804583334</v>
       </c>
       <c r="Q74" s="8">
         <v>1</v>
@@ -5814,7 +5814,7 @@
         <v>46315.417349537034</v>
       </c>
       <c r="P75" s="3">
-        <v>46317.51144902778</v>
+        <v>46317.531804583334</v>
       </c>
       <c r="Q75" s="8">
         <v>0</v>
@@ -5886,7 +5886,7 @@
         <v>46315.417349537034</v>
       </c>
       <c r="P76" s="3">
-        <v>46317.51144824074</v>
+        <v>46317.53180380787</v>
       </c>
       <c r="Q76" s="8">
         <v>0</v>
@@ -5963,7 +5963,7 @@
         <v>46315.417129629626</v>
       </c>
       <c r="P77" s="3">
-        <v>46317.5114486574</v>
+        <v>46317.53180420139</v>
       </c>
       <c r="Q77" s="8">
         <v>0</v>
@@ -6040,7 +6040,7 @@
         <v>46315.41690972222</v>
       </c>
       <c r="P78" s="3">
-        <v>46317.5114486574</v>
+        <v>46317.53180420139</v>
       </c>
       <c r="Q78" s="8">
         <v>0</v>
@@ -6117,7 +6117,7 @@
         <v>46315.41668981481</v>
       </c>
       <c r="P79" s="3">
-        <v>46317.5114486574</v>
+        <v>46317.53180420139</v>
       </c>
       <c r="Q79" s="8">
         <v>0</v>
@@ -6194,7 +6194,7 @@
         <v>46315.41716435185</v>
       </c>
       <c r="P80" s="3">
-        <v>46317.51154056713</v>
+        <v>46317.53189219907</v>
       </c>
       <c r="Q80" s="8">
         <v>0</v>
@@ -6271,7 +6271,7 @@
         <v>46315.41694444444</v>
       </c>
       <c r="P81" s="3">
-        <v>46317.51144902778</v>
+        <v>46317.531804583334</v>
       </c>
       <c r="Q81" s="8">
         <v>1</v>
@@ -6348,7 +6348,7 @@
         <v>46315.41672453703</v>
       </c>
       <c r="P82" s="3">
-        <v>46317.51144824074</v>
+        <v>46317.53180380787</v>
       </c>
       <c r="Q82" s="8">
         <v>0</v>
@@ -6425,7 +6425,7 @@
         <v>46315.41719907407</v>
       </c>
       <c r="P83" s="3">
-        <v>46317.51154056713</v>
+        <v>46317.53189219907</v>
       </c>
       <c r="Q83" s="8">
         <v>0</v>
@@ -6497,7 +6497,7 @@
         <v>46315.416979166665</v>
       </c>
       <c r="P84" s="3">
-        <v>46317.5114486574</v>
+        <v>46317.53180420139</v>
       </c>
       <c r="Q84" s="8">
         <v>0</v>
@@ -6574,7 +6574,7 @@
         <v>46315.41675925926</v>
       </c>
       <c r="P85" s="3">
-        <v>46317.5114486574</v>
+        <v>46317.53180420139</v>
       </c>
       <c r="Q85" s="8">
         <v>0</v>
@@ -6651,7 +6651,7 @@
         <v>46315.417233796295</v>
       </c>
       <c r="P86" s="3">
-        <v>46317.51144902778</v>
+        <v>46317.531804583334</v>
       </c>
       <c r="Q86" s="8">
         <v>0</v>
@@ -6728,7 +6728,7 @@
         <v>46315.41701388889</v>
       </c>
       <c r="P87" s="3">
-        <v>46317.51144902778</v>
+        <v>46317.531804583334</v>
       </c>
       <c r="Q87" s="8">
         <v>3</v>
@@ -6805,7 +6805,7 @@
         <v>46315.41679398148</v>
       </c>
       <c r="P88" s="3">
-        <v>46317.51144824074</v>
+        <v>46317.53180380787</v>
       </c>
       <c r="Q88" s="8">
         <v>0</v>
@@ -6882,7 +6882,7 @@
         <v>46315.41726851852</v>
       </c>
       <c r="P89" s="3">
-        <v>46317.5114486574</v>
+        <v>46317.53180420139</v>
       </c>
       <c r="Q89" s="8">
         <v>0</v>
@@ -6959,7 +6959,7 @@
         <v>46315.41704861111</v>
       </c>
       <c r="P90" s="3">
-        <v>46317.5114486574</v>
+        <v>46317.53180420139</v>
       </c>
       <c r="Q90" s="8">
         <v>0</v>
@@ -7036,7 +7036,7 @@
         <v>46315.4168287037</v>
       </c>
       <c r="P91" s="3">
-        <v>46317.5114486574</v>
+        <v>46317.53180420139</v>
       </c>
       <c r="Q91" s="8">
         <v>0</v>
@@ -7108,7 +7108,7 @@
         <v>46315.41730324074</v>
       </c>
       <c r="P92" s="3">
-        <v>46317.51144902778</v>
+        <v>46317.531804583334</v>
       </c>
       <c r="Q92" s="8">
         <v>0</v>
@@ -7185,7 +7185,7 @@
         <v>46315.417083333334</v>
       </c>
       <c r="P93" s="3">
-        <v>46317.51144902778</v>
+        <v>46317.531804583334</v>
       </c>
       <c r="Q93" s="8">
         <v>1</v>
@@ -7262,7 +7262,7 @@
         <v>46315.416863425926</v>
       </c>
       <c r="P94" s="3">
-        <v>46317.51144824074</v>
+        <v>46317.53180380787</v>
       </c>
       <c r="Q94" s="8">
         <v>0</v>
@@ -7339,7 +7339,7 @@
         <v>46315.417337962965</v>
       </c>
       <c r="P95" s="3">
-        <v>46317.5114486574</v>
+        <v>46317.53180420139</v>
       </c>
       <c r="Q95" s="8">
         <v>0</v>
@@ -7416,7 +7416,7 @@
         <v>46315.41711805556</v>
       </c>
       <c r="P96" s="3">
-        <v>46317.5114486574</v>
+        <v>46317.53180420139</v>
       </c>
       <c r="Q96" s="8">
         <v>0</v>
@@ -7493,7 +7493,7 @@
         <v>46315.41689814815</v>
       </c>
       <c r="P97" s="3">
-        <v>46317.51144902778</v>
+        <v>46317.531804583334</v>
       </c>
       <c r="Q97" s="8">
         <v>0</v>
@@ -7570,7 +7570,7 @@
         <v>46315.41667824074</v>
       </c>
       <c r="P98" s="3">
-        <v>46317.51154056713</v>
+        <v>46317.53189219907</v>
       </c>
       <c r="Q98" s="8">
         <v>0</v>
@@ -7647,7 +7647,7 @@
         <v>46315.41715277778</v>
       </c>
       <c r="P99" s="3">
-        <v>46317.51144902778</v>
+        <v>46317.531804583334</v>
       </c>
       <c r="Q99" s="8">
         <v>1</v>
@@ -7719,7 +7719,7 @@
         <v>46315.41693287037</v>
       </c>
       <c r="P100" s="3">
-        <v>46317.51144824074</v>
+        <v>46317.53180380787</v>
       </c>
       <c r="Q100" s="8">
         <v>0</v>
@@ -7796,7 +7796,7 @@
         <v>46315.416712962964</v>
       </c>
       <c r="P101" s="3">
-        <v>46317.51154056713</v>
+        <v>46317.53189219907</v>
       </c>
       <c r="Q101" s="8">
         <v>0</v>
@@ -7873,7 +7873,7 @@
         <v>46315.4171875</v>
       </c>
       <c r="P102" s="3">
-        <v>46317.5114486574</v>
+        <v>46317.53180420139</v>
       </c>
       <c r="Q102" s="8">
         <v>3</v>
@@ -7950,7 +7950,7 @@
         <v>46315.416967592595</v>
       </c>
       <c r="P103" s="3">
-        <v>46317.51144902778</v>
+        <v>46317.531804583334</v>
       </c>
       <c r="Q103" s="8">
         <v>0</v>
@@ -8027,7 +8027,7 @@
         <v>46315.41674768519</v>
       </c>
       <c r="P104" s="3">
-        <v>46317.51144902778</v>
+        <v>46317.531804583334</v>
       </c>
       <c r="Q104" s="8">
         <v>0</v>
@@ -8104,7 +8104,7 @@
         <v>46315.417222222226</v>
       </c>
       <c r="P105" s="3">
-        <v>46317.51144902778</v>
+        <v>46317.531804583334</v>
       </c>
       <c r="Q105" s="8">
         <v>1</v>
@@ -8181,7 +8181,7 @@
         <v>46315.41700231482</v>
       </c>
       <c r="P106" s="3">
-        <v>46317.51144824074</v>
+        <v>46317.53180380787</v>
       </c>
       <c r="Q106" s="8">
         <v>0</v>
@@ -8258,7 +8258,7 @@
         <v>46315.41678240741</v>
       </c>
       <c r="P107" s="3">
-        <v>46317.5114486574</v>
+        <v>46317.53180420139</v>
       </c>
       <c r="Q107" s="8">
         <v>0</v>
@@ -8330,7 +8330,7 @@
         <v>46315.41725694445</v>
       </c>
       <c r="P108" s="3">
-        <v>46317.5114486574</v>
+        <v>46317.53180420139</v>
       </c>
       <c r="Q108" s="8">
         <v>0</v>
@@ -8407,7 +8407,7 @@
         <v>46315.41703703704</v>
       </c>
       <c r="P109" s="3">
-        <v>46317.51144902778</v>
+        <v>46317.531804583334</v>
       </c>
       <c r="Q109" s="8">
         <v>0</v>
@@ -8484,7 +8484,7 @@
         <v>46315.41681712963</v>
       </c>
       <c r="P110" s="3">
-        <v>46317.51144902778</v>
+        <v>46317.531804583334</v>
       </c>
       <c r="Q110" s="8">
         <v>0</v>
@@ -8561,7 +8561,7 @@
         <v>46315.41729166667</v>
       </c>
       <c r="P111" s="3">
-        <v>46317.51144902778</v>
+        <v>46317.531804583334</v>
       </c>
       <c r="Q111" s="8">
         <v>1</v>
@@ -8633,7 +8633,7 @@
         <v>46315.41729166667</v>
       </c>
       <c r="P112" s="3">
-        <v>46317.51144824074</v>
+        <v>46317.53180380787</v>
       </c>
       <c r="Q112" s="8">
         <v>1</v>
@@ -8705,7 +8705,7 @@
         <v>46315.417071759264</v>
       </c>
       <c r="P113" s="3">
-        <v>46317.51144824074</v>
+        <v>46317.53180380787</v>
       </c>
       <c r="Q113" s="8">
         <v>0</v>
@@ -8777,7 +8777,7 @@
         <v>46315.416851851856</v>
       </c>
       <c r="P114" s="3">
-        <v>46317.5114486574</v>
+        <v>46317.53180420139</v>
       </c>
       <c r="Q114" s="8">
         <v>0</v>
@@ -8849,7 +8849,7 @@
         <v>46315.41732638889</v>
       </c>
       <c r="P115" s="3">
-        <v>46317.5114486574</v>
+        <v>46317.53180420139</v>
       </c>
       <c r="Q115" s="8">
         <v>0</v>
@@ -8921,7 +8921,7 @@
         <v>46315.41710648148</v>
       </c>
       <c r="P116" s="3">
-        <v>46317.51144902778</v>
+        <v>46317.531804583334</v>
       </c>
       <c r="Q116" s="8">
         <v>0</v>
@@ -8988,7 +8988,7 @@
         <v>46315.41688657408</v>
       </c>
       <c r="P117" s="3">
-        <v>46317.51154056713</v>
+        <v>46317.53189219907</v>
       </c>
       <c r="Q117" s="8">
         <v>0</v>

</xml_diff>

<commit_message>
Capture header: project selector in top bar, remove project card and All Projects link, compact tour row
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/poc-output/m9-chromium/export-filtered.xlsx
+++ b/poc-output/m9-chromium/export-filtered.xlsx
@@ -293,7 +293,7 @@
         <v>46315.41677083333</v>
       </c>
       <c r="P2" s="3">
-        <v>46317.53180380787</v>
+        <v>46317.53738854166</v>
       </c>
       <c r="Q2" s="8">
         <v>0</v>
@@ -365,7 +365,7 @@
         <v>46315.417245370365</v>
       </c>
       <c r="P3" s="3">
-        <v>46317.53180420139</v>
+        <v>46317.53738892361</v>
       </c>
       <c r="Q3" s="8">
         <v>0</v>
@@ -437,7 +437,7 @@
         <v>46315.417025462964</v>
       </c>
       <c r="P4" s="3">
-        <v>46317.53189219907</v>
+        <v>46317.53747668982</v>
       </c>
       <c r="Q4" s="8">
         <v>0</v>
@@ -509,7 +509,7 @@
         <v>46315.41680555556</v>
       </c>
       <c r="P5" s="3">
-        <v>46317.53180420139</v>
+        <v>46317.53738892361</v>
       </c>
       <c r="Q5" s="8">
         <v>1</v>
@@ -581,7 +581,7 @@
         <v>46315.41728009259</v>
       </c>
       <c r="P6" s="3">
-        <v>46317.531876574074</v>
+        <v>46317.53746143519</v>
       </c>
       <c r="Q6" s="8">
         <v>0</v>
@@ -653,7 +653,7 @@
         <v>46315.41706018518</v>
       </c>
       <c r="P7" s="3">
-        <v>46317.531804583334</v>
+        <v>46317.537389317135</v>
       </c>
       <c r="Q7" s="8">
         <v>0</v>
@@ -720,7 +720,7 @@
         <v>46315.41684027778</v>
       </c>
       <c r="P8" s="3">
-        <v>46317.53180380787</v>
+        <v>46317.53738854166</v>
       </c>
       <c r="Q8" s="8">
         <v>3</v>
@@ -792,7 +792,7 @@
         <v>46315.41731481481</v>
       </c>
       <c r="P9" s="3">
-        <v>46317.531876574074</v>
+        <v>46317.53746143519</v>
       </c>
       <c r="Q9" s="8">
         <v>0</v>
@@ -864,7 +864,7 @@
         <v>46315.4170949074</v>
       </c>
       <c r="P10" s="3">
-        <v>46317.53180420139</v>
+        <v>46317.53738892361</v>
       </c>
       <c r="Q10" s="8">
         <v>0</v>
@@ -936,7 +936,7 @@
         <v>46315.416874999995</v>
       </c>
       <c r="P11" s="3">
-        <v>46317.53180420139</v>
+        <v>46317.53738892361</v>
       </c>
       <c r="Q11" s="8">
         <v>1</v>
@@ -1008,7 +1008,7 @@
         <v>46315.417349537034</v>
       </c>
       <c r="P12" s="3">
-        <v>46317.531804583334</v>
+        <v>46317.537389317135</v>
       </c>
       <c r="Q12" s="8">
         <v>0</v>
@@ -1080,7 +1080,7 @@
         <v>46315.417129629626</v>
       </c>
       <c r="P13" s="3">
-        <v>46317.531804583334</v>
+        <v>46317.537389317135</v>
       </c>
       <c r="Q13" s="8">
         <v>0</v>
@@ -1157,7 +1157,7 @@
         <v>46315.41690972222</v>
       </c>
       <c r="P14" s="3">
-        <v>46317.53180380787</v>
+        <v>46317.53738854166</v>
       </c>
       <c r="Q14" s="8">
         <v>0</v>
@@ -1234,7 +1234,7 @@
         <v>46315.41668981481</v>
       </c>
       <c r="P15" s="3">
-        <v>46317.53180420139</v>
+        <v>46317.53738892361</v>
       </c>
       <c r="Q15" s="8">
         <v>0</v>
@@ -1306,7 +1306,7 @@
         <v>46315.41716435185</v>
       </c>
       <c r="P16" s="3">
-        <v>46317.53180420139</v>
+        <v>46317.53738892361</v>
       </c>
       <c r="Q16" s="8">
         <v>0</v>
@@ -1383,7 +1383,7 @@
         <v>46315.41694444444</v>
       </c>
       <c r="P17" s="3">
-        <v>46317.531804583334</v>
+        <v>46317.537389317135</v>
       </c>
       <c r="Q17" s="8">
         <v>1</v>
@@ -1460,7 +1460,7 @@
         <v>46315.41672453703</v>
       </c>
       <c r="P18" s="3">
-        <v>46317.531804583334</v>
+        <v>46317.537389317135</v>
       </c>
       <c r="Q18" s="8">
         <v>0</v>
@@ -1537,7 +1537,7 @@
         <v>46315.41719907407</v>
       </c>
       <c r="P19" s="3">
-        <v>46317.53189219907</v>
+        <v>46317.53747668982</v>
       </c>
       <c r="Q19" s="8">
         <v>0</v>
@@ -1614,7 +1614,7 @@
         <v>46315.416979166665</v>
       </c>
       <c r="P20" s="3">
-        <v>46317.53180380787</v>
+        <v>46317.53738854166</v>
       </c>
       <c r="Q20" s="8">
         <v>0</v>
@@ -1691,7 +1691,7 @@
         <v>46315.41675925926</v>
       </c>
       <c r="P21" s="3">
-        <v>46317.53180420139</v>
+        <v>46317.53738892361</v>
       </c>
       <c r="Q21" s="8">
         <v>0</v>
@@ -1768,7 +1768,7 @@
         <v>46315.417233796295</v>
       </c>
       <c r="P22" s="3">
-        <v>46317.53189219907</v>
+        <v>46317.53747668982</v>
       </c>
       <c r="Q22" s="8">
         <v>0</v>
@@ -1845,7 +1845,7 @@
         <v>46315.41701388889</v>
       </c>
       <c r="P23" s="3">
-        <v>46317.531804583334</v>
+        <v>46317.537389317135</v>
       </c>
       <c r="Q23" s="8">
         <v>3</v>
@@ -1917,7 +1917,7 @@
         <v>46315.41679398148</v>
       </c>
       <c r="P24" s="3">
-        <v>46317.531876574074</v>
+        <v>46317.53746143519</v>
       </c>
       <c r="Q24" s="8">
         <v>0</v>
@@ -1994,7 +1994,7 @@
         <v>46315.41726851852</v>
       </c>
       <c r="P25" s="3">
-        <v>46317.531804583334</v>
+        <v>46317.537389317135</v>
       </c>
       <c r="Q25" s="8">
         <v>0</v>
@@ -2071,7 +2071,7 @@
         <v>46315.41726851852</v>
       </c>
       <c r="P26" s="3">
-        <v>46317.53189219907</v>
+        <v>46317.53747668982</v>
       </c>
       <c r="Q26" s="8">
         <v>0</v>
@@ -2148,7 +2148,7 @@
         <v>46315.41704861111</v>
       </c>
       <c r="P27" s="3">
-        <v>46317.53180380787</v>
+        <v>46317.53738854166</v>
       </c>
       <c r="Q27" s="8">
         <v>0</v>
@@ -2225,7 +2225,7 @@
         <v>46315.4168287037</v>
       </c>
       <c r="P28" s="3">
-        <v>46317.531876574074</v>
+        <v>46317.53746143519</v>
       </c>
       <c r="Q28" s="8">
         <v>0</v>
@@ -2302,7 +2302,7 @@
         <v>46315.41730324074</v>
       </c>
       <c r="P29" s="3">
-        <v>46317.53180420139</v>
+        <v>46317.53738892361</v>
       </c>
       <c r="Q29" s="8">
         <v>0</v>
@@ -2379,7 +2379,7 @@
         <v>46315.417083333334</v>
       </c>
       <c r="P30" s="3">
-        <v>46317.531804583334</v>
+        <v>46317.537389317135</v>
       </c>
       <c r="Q30" s="8">
         <v>1</v>
@@ -2456,7 +2456,7 @@
         <v>46315.416863425926</v>
       </c>
       <c r="P31" s="3">
-        <v>46317.531804583334</v>
+        <v>46317.537389317135</v>
       </c>
       <c r="Q31" s="8">
         <v>0</v>
@@ -2533,7 +2533,7 @@
         <v>46315.417337962965</v>
       </c>
       <c r="P32" s="3">
-        <v>46317.531804583334</v>
+        <v>46317.537389317135</v>
       </c>
       <c r="Q32" s="8">
         <v>0</v>
@@ -2610,7 +2610,7 @@
         <v>46315.417337962965</v>
       </c>
       <c r="P33" s="3">
-        <v>46317.53180380787</v>
+        <v>46317.53738854166</v>
       </c>
       <c r="Q33" s="8">
         <v>0</v>
@@ -2682,7 +2682,7 @@
         <v>46315.41711805556</v>
       </c>
       <c r="P34" s="3">
-        <v>46317.53180380787</v>
+        <v>46317.53738854166</v>
       </c>
       <c r="Q34" s="8">
         <v>0</v>
@@ -2759,7 +2759,7 @@
         <v>46315.41689814815</v>
       </c>
       <c r="P35" s="3">
-        <v>46317.53180420139</v>
+        <v>46317.53738892361</v>
       </c>
       <c r="Q35" s="8">
         <v>0</v>
@@ -2836,7 +2836,7 @@
         <v>46315.41667824074</v>
       </c>
       <c r="P36" s="3">
-        <v>46317.53180420139</v>
+        <v>46317.53738892361</v>
       </c>
       <c r="Q36" s="8">
         <v>0</v>
@@ -2913,7 +2913,7 @@
         <v>46315.41715277778</v>
       </c>
       <c r="P37" s="3">
-        <v>46317.531804583334</v>
+        <v>46317.537389317135</v>
       </c>
       <c r="Q37" s="8">
         <v>1</v>
@@ -2990,7 +2990,7 @@
         <v>46315.41693287037</v>
       </c>
       <c r="P38" s="3">
-        <v>46317.531804583334</v>
+        <v>46317.537389317135</v>
       </c>
       <c r="Q38" s="8">
         <v>0</v>
@@ -3067,7 +3067,7 @@
         <v>46315.416712962964</v>
       </c>
       <c r="P39" s="3">
-        <v>46317.53180380787</v>
+        <v>46317.53738854166</v>
       </c>
       <c r="Q39" s="8">
         <v>0</v>
@@ -3144,7 +3144,7 @@
         <v>46315.4171875</v>
       </c>
       <c r="P40" s="3">
-        <v>46317.53180420139</v>
+        <v>46317.53738892361</v>
       </c>
       <c r="Q40" s="8">
         <v>3</v>
@@ -3221,7 +3221,7 @@
         <v>46315.416967592595</v>
       </c>
       <c r="P41" s="3">
-        <v>46317.53180420139</v>
+        <v>46317.53738892361</v>
       </c>
       <c r="Q41" s="8">
         <v>0</v>
@@ -3293,7 +3293,7 @@
         <v>46315.41674768519</v>
       </c>
       <c r="P42" s="3">
-        <v>46317.53189219907</v>
+        <v>46317.53747668982</v>
       </c>
       <c r="Q42" s="8">
         <v>0</v>
@@ -3370,7 +3370,7 @@
         <v>46315.417222222226</v>
       </c>
       <c r="P43" s="3">
-        <v>46317.531804583334</v>
+        <v>46317.537389317135</v>
       </c>
       <c r="Q43" s="8">
         <v>1</v>
@@ -3447,7 +3447,7 @@
         <v>46315.41700231482</v>
       </c>
       <c r="P44" s="3">
-        <v>46317.531804583334</v>
+        <v>46317.537389317135</v>
       </c>
       <c r="Q44" s="8">
         <v>0</v>
@@ -3524,7 +3524,7 @@
         <v>46315.41678240741</v>
       </c>
       <c r="P45" s="3">
-        <v>46317.53189219907</v>
+        <v>46317.53747668982</v>
       </c>
       <c r="Q45" s="8">
         <v>0</v>
@@ -3601,7 +3601,7 @@
         <v>46315.41725694445</v>
       </c>
       <c r="P46" s="3">
-        <v>46317.53180420139</v>
+        <v>46317.53738892361</v>
       </c>
       <c r="Q46" s="8">
         <v>0</v>
@@ -3678,7 +3678,7 @@
         <v>46315.41703703704</v>
       </c>
       <c r="P47" s="3">
-        <v>46317.53180420139</v>
+        <v>46317.53738892361</v>
       </c>
       <c r="Q47" s="8">
         <v>0</v>
@@ -3755,7 +3755,7 @@
         <v>46315.41681712963</v>
       </c>
       <c r="P48" s="3">
-        <v>46317.53180420139</v>
+        <v>46317.53738892361</v>
       </c>
       <c r="Q48" s="8">
         <v>0</v>
@@ -3832,7 +3832,7 @@
         <v>46315.41729166667</v>
       </c>
       <c r="P49" s="3">
-        <v>46317.531804583334</v>
+        <v>46317.537389317135</v>
       </c>
       <c r="Q49" s="8">
         <v>1</v>
@@ -3904,7 +3904,7 @@
         <v>46315.417071759264</v>
       </c>
       <c r="P50" s="3">
-        <v>46317.531804583334</v>
+        <v>46317.537389317135</v>
       </c>
       <c r="Q50" s="8">
         <v>0</v>
@@ -3981,7 +3981,7 @@
         <v>46315.416851851856</v>
       </c>
       <c r="P51" s="3">
-        <v>46317.53180380787</v>
+        <v>46317.53738854166</v>
       </c>
       <c r="Q51" s="8">
         <v>0</v>
@@ -4058,7 +4058,7 @@
         <v>46315.41732638889</v>
       </c>
       <c r="P52" s="3">
-        <v>46317.53180420139</v>
+        <v>46317.53738892361</v>
       </c>
       <c r="Q52" s="8">
         <v>0</v>
@@ -4135,7 +4135,7 @@
         <v>46315.41710648148</v>
       </c>
       <c r="P53" s="3">
-        <v>46317.53180420139</v>
+        <v>46317.53738892361</v>
       </c>
       <c r="Q53" s="8">
         <v>0</v>
@@ -4212,7 +4212,7 @@
         <v>46315.41688657408</v>
       </c>
       <c r="P54" s="3">
-        <v>46317.53180420139</v>
+        <v>46317.53738892361</v>
       </c>
       <c r="Q54" s="8">
         <v>0</v>
@@ -4289,7 +4289,7 @@
         <v>46315.41666666667</v>
       </c>
       <c r="P55" s="3">
-        <v>46317.531804583334</v>
+        <v>46317.537389317135</v>
       </c>
       <c r="Q55" s="8">
         <v>3</v>
@@ -4366,7 +4366,7 @@
         <v>46315.4171412037</v>
       </c>
       <c r="P56" s="3">
-        <v>46317.531804583334</v>
+        <v>46317.537389317135</v>
       </c>
       <c r="Q56" s="8">
         <v>0</v>
@@ -4443,7 +4443,7 @@
         <v>46315.416921296295</v>
       </c>
       <c r="P57" s="3">
-        <v>46317.53180380787</v>
+        <v>46317.53738854166</v>
       </c>
       <c r="Q57" s="8">
         <v>0</v>
@@ -4515,7 +4515,7 @@
         <v>46315.41670138889</v>
       </c>
       <c r="P58" s="3">
-        <v>46317.53180420139</v>
+        <v>46317.53738892361</v>
       </c>
       <c r="Q58" s="8">
         <v>0</v>
@@ -4592,7 +4592,7 @@
         <v>46315.417175925926</v>
       </c>
       <c r="P59" s="3">
-        <v>46317.53180420139</v>
+        <v>46317.53738892361</v>
       </c>
       <c r="Q59" s="8">
         <v>0</v>
@@ -4669,7 +4669,7 @@
         <v>46315.41695601852</v>
       </c>
       <c r="P60" s="3">
-        <v>46317.53189219907</v>
+        <v>46317.53747668982</v>
       </c>
       <c r="Q60" s="8">
         <v>0</v>
@@ -4746,7 +4746,7 @@
         <v>46315.41673611111</v>
       </c>
       <c r="P61" s="3">
-        <v>46317.531804583334</v>
+        <v>46317.537389317135</v>
       </c>
       <c r="Q61" s="8">
         <v>1</v>
@@ -4823,7 +4823,7 @@
         <v>46315.41721064815</v>
       </c>
       <c r="P62" s="3">
-        <v>46317.531876574074</v>
+        <v>46317.53746143519</v>
       </c>
       <c r="Q62" s="8">
         <v>0</v>
@@ -4900,7 +4900,7 @@
         <v>46315.41699074074</v>
       </c>
       <c r="P63" s="3">
-        <v>46317.53189219907</v>
+        <v>46317.53747668982</v>
       </c>
       <c r="Q63" s="8">
         <v>0</v>
@@ -4977,7 +4977,7 @@
         <v>46315.41677083333</v>
       </c>
       <c r="P64" s="3">
-        <v>46317.53180420139</v>
+        <v>46317.53738892361</v>
       </c>
       <c r="Q64" s="8">
         <v>0</v>
@@ -5054,7 +5054,7 @@
         <v>46315.417245370365</v>
       </c>
       <c r="P65" s="3">
-        <v>46317.531876574074</v>
+        <v>46317.53746143519</v>
       </c>
       <c r="Q65" s="8">
         <v>0</v>
@@ -5126,7 +5126,7 @@
         <v>46315.417025462964</v>
       </c>
       <c r="P66" s="3">
-        <v>46317.531804583334</v>
+        <v>46317.537389317135</v>
       </c>
       <c r="Q66" s="8">
         <v>0</v>
@@ -5203,7 +5203,7 @@
         <v>46315.41680555556</v>
       </c>
       <c r="P67" s="3">
-        <v>46317.531804583334</v>
+        <v>46317.537389317135</v>
       </c>
       <c r="Q67" s="8">
         <v>1</v>
@@ -5280,7 +5280,7 @@
         <v>46315.41728009259</v>
       </c>
       <c r="P68" s="3">
-        <v>46317.531804583334</v>
+        <v>46317.537389317135</v>
       </c>
       <c r="Q68" s="8">
         <v>0</v>
@@ -5357,7 +5357,7 @@
         <v>46315.41728009259</v>
       </c>
       <c r="P69" s="3">
-        <v>46317.531876574074</v>
+        <v>46317.53746143519</v>
       </c>
       <c r="Q69" s="8">
         <v>0</v>
@@ -5434,7 +5434,7 @@
         <v>46315.41706018518</v>
       </c>
       <c r="P70" s="3">
-        <v>46317.53180380787</v>
+        <v>46317.53738854166</v>
       </c>
       <c r="Q70" s="8">
         <v>0</v>
@@ -5511,7 +5511,7 @@
         <v>46315.41684027778</v>
       </c>
       <c r="P71" s="3">
-        <v>46317.53180420139</v>
+        <v>46317.53738892361</v>
       </c>
       <c r="Q71" s="8">
         <v>3</v>
@@ -5588,7 +5588,7 @@
         <v>46315.41731481481</v>
       </c>
       <c r="P72" s="3">
-        <v>46317.53180420139</v>
+        <v>46317.53738892361</v>
       </c>
       <c r="Q72" s="8">
         <v>0</v>
@@ -5665,7 +5665,7 @@
         <v>46315.4170949074</v>
       </c>
       <c r="P73" s="3">
-        <v>46317.531804583334</v>
+        <v>46317.537389317135</v>
       </c>
       <c r="Q73" s="8">
         <v>0</v>
@@ -5742,7 +5742,7 @@
         <v>46315.416874999995</v>
       </c>
       <c r="P74" s="3">
-        <v>46317.531804583334</v>
+        <v>46317.537389317135</v>
       </c>
       <c r="Q74" s="8">
         <v>1</v>
@@ -5814,7 +5814,7 @@
         <v>46315.417349537034</v>
       </c>
       <c r="P75" s="3">
-        <v>46317.531804583334</v>
+        <v>46317.537389317135</v>
       </c>
       <c r="Q75" s="8">
         <v>0</v>
@@ -5886,7 +5886,7 @@
         <v>46315.417349537034</v>
       </c>
       <c r="P76" s="3">
-        <v>46317.53180380787</v>
+        <v>46317.53738854166</v>
       </c>
       <c r="Q76" s="8">
         <v>0</v>
@@ -5963,7 +5963,7 @@
         <v>46315.417129629626</v>
       </c>
       <c r="P77" s="3">
-        <v>46317.53180420139</v>
+        <v>46317.53738892361</v>
       </c>
       <c r="Q77" s="8">
         <v>0</v>
@@ -6040,7 +6040,7 @@
         <v>46315.41690972222</v>
       </c>
       <c r="P78" s="3">
-        <v>46317.53180420139</v>
+        <v>46317.53738892361</v>
       </c>
       <c r="Q78" s="8">
         <v>0</v>
@@ -6117,7 +6117,7 @@
         <v>46315.41668981481</v>
       </c>
       <c r="P79" s="3">
-        <v>46317.53180420139</v>
+        <v>46317.53738892361</v>
       </c>
       <c r="Q79" s="8">
         <v>0</v>
@@ -6194,7 +6194,7 @@
         <v>46315.41716435185</v>
       </c>
       <c r="P80" s="3">
-        <v>46317.53189219907</v>
+        <v>46317.53747668982</v>
       </c>
       <c r="Q80" s="8">
         <v>0</v>
@@ -6271,7 +6271,7 @@
         <v>46315.41694444444</v>
       </c>
       <c r="P81" s="3">
-        <v>46317.531804583334</v>
+        <v>46317.537389317135</v>
       </c>
       <c r="Q81" s="8">
         <v>1</v>
@@ -6348,7 +6348,7 @@
         <v>46315.41672453703</v>
       </c>
       <c r="P82" s="3">
-        <v>46317.53180380787</v>
+        <v>46317.53738854166</v>
       </c>
       <c r="Q82" s="8">
         <v>0</v>
@@ -6425,7 +6425,7 @@
         <v>46315.41719907407</v>
       </c>
       <c r="P83" s="3">
-        <v>46317.53189219907</v>
+        <v>46317.53747668982</v>
       </c>
       <c r="Q83" s="8">
         <v>0</v>
@@ -6497,7 +6497,7 @@
         <v>46315.416979166665</v>
       </c>
       <c r="P84" s="3">
-        <v>46317.53180420139</v>
+        <v>46317.53738892361</v>
       </c>
       <c r="Q84" s="8">
         <v>0</v>
@@ -6574,7 +6574,7 @@
         <v>46315.41675925926</v>
       </c>
       <c r="P85" s="3">
-        <v>46317.53180420139</v>
+        <v>46317.53738892361</v>
       </c>
       <c r="Q85" s="8">
         <v>0</v>
@@ -6651,7 +6651,7 @@
         <v>46315.417233796295</v>
       </c>
       <c r="P86" s="3">
-        <v>46317.531804583334</v>
+        <v>46317.537389317135</v>
       </c>
       <c r="Q86" s="8">
         <v>0</v>
@@ -6728,7 +6728,7 @@
         <v>46315.41701388889</v>
       </c>
       <c r="P87" s="3">
-        <v>46317.531804583334</v>
+        <v>46317.537389317135</v>
       </c>
       <c r="Q87" s="8">
         <v>3</v>
@@ -6805,7 +6805,7 @@
         <v>46315.41679398148</v>
       </c>
       <c r="P88" s="3">
-        <v>46317.53180380787</v>
+        <v>46317.53738854166</v>
       </c>
       <c r="Q88" s="8">
         <v>0</v>
@@ -6882,7 +6882,7 @@
         <v>46315.41726851852</v>
       </c>
       <c r="P89" s="3">
-        <v>46317.53180420139</v>
+        <v>46317.53738892361</v>
       </c>
       <c r="Q89" s="8">
         <v>0</v>
@@ -6959,7 +6959,7 @@
         <v>46315.41704861111</v>
       </c>
       <c r="P90" s="3">
-        <v>46317.53180420139</v>
+        <v>46317.53738892361</v>
       </c>
       <c r="Q90" s="8">
         <v>0</v>
@@ -7036,7 +7036,7 @@
         <v>46315.4168287037</v>
       </c>
       <c r="P91" s="3">
-        <v>46317.53180420139</v>
+        <v>46317.53738892361</v>
       </c>
       <c r="Q91" s="8">
         <v>0</v>
@@ -7108,7 +7108,7 @@
         <v>46315.41730324074</v>
       </c>
       <c r="P92" s="3">
-        <v>46317.531804583334</v>
+        <v>46317.537389317135</v>
       </c>
       <c r="Q92" s="8">
         <v>0</v>
@@ -7185,7 +7185,7 @@
         <v>46315.417083333334</v>
       </c>
       <c r="P93" s="3">
-        <v>46317.531804583334</v>
+        <v>46317.537389317135</v>
       </c>
       <c r="Q93" s="8">
         <v>1</v>
@@ -7262,7 +7262,7 @@
         <v>46315.416863425926</v>
       </c>
       <c r="P94" s="3">
-        <v>46317.53180380787</v>
+        <v>46317.53738854166</v>
       </c>
       <c r="Q94" s="8">
         <v>0</v>
@@ -7339,7 +7339,7 @@
         <v>46315.417337962965</v>
       </c>
       <c r="P95" s="3">
-        <v>46317.53180420139</v>
+        <v>46317.53738892361</v>
       </c>
       <c r="Q95" s="8">
         <v>0</v>
@@ -7416,7 +7416,7 @@
         <v>46315.41711805556</v>
       </c>
       <c r="P96" s="3">
-        <v>46317.53180420139</v>
+        <v>46317.53738892361</v>
       </c>
       <c r="Q96" s="8">
         <v>0</v>
@@ -7493,7 +7493,7 @@
         <v>46315.41689814815</v>
       </c>
       <c r="P97" s="3">
-        <v>46317.531804583334</v>
+        <v>46317.537389317135</v>
       </c>
       <c r="Q97" s="8">
         <v>0</v>
@@ -7570,7 +7570,7 @@
         <v>46315.41667824074</v>
       </c>
       <c r="P98" s="3">
-        <v>46317.53189219907</v>
+        <v>46317.53747668982</v>
       </c>
       <c r="Q98" s="8">
         <v>0</v>
@@ -7647,7 +7647,7 @@
         <v>46315.41715277778</v>
       </c>
       <c r="P99" s="3">
-        <v>46317.531804583334</v>
+        <v>46317.537389317135</v>
       </c>
       <c r="Q99" s="8">
         <v>1</v>
@@ -7719,7 +7719,7 @@
         <v>46315.41693287037</v>
       </c>
       <c r="P100" s="3">
-        <v>46317.53180380787</v>
+        <v>46317.53738854166</v>
       </c>
       <c r="Q100" s="8">
         <v>0</v>
@@ -7796,7 +7796,7 @@
         <v>46315.416712962964</v>
       </c>
       <c r="P101" s="3">
-        <v>46317.53189219907</v>
+        <v>46317.53747668982</v>
       </c>
       <c r="Q101" s="8">
         <v>0</v>
@@ -7873,7 +7873,7 @@
         <v>46315.4171875</v>
       </c>
       <c r="P102" s="3">
-        <v>46317.53180420139</v>
+        <v>46317.53738892361</v>
       </c>
       <c r="Q102" s="8">
         <v>3</v>
@@ -7950,7 +7950,7 @@
         <v>46315.416967592595</v>
       </c>
       <c r="P103" s="3">
-        <v>46317.531804583334</v>
+        <v>46317.537389317135</v>
       </c>
       <c r="Q103" s="8">
         <v>0</v>
@@ -8027,7 +8027,7 @@
         <v>46315.41674768519</v>
       </c>
       <c r="P104" s="3">
-        <v>46317.531804583334</v>
+        <v>46317.537389317135</v>
       </c>
       <c r="Q104" s="8">
         <v>0</v>
@@ -8104,7 +8104,7 @@
         <v>46315.417222222226</v>
       </c>
       <c r="P105" s="3">
-        <v>46317.531804583334</v>
+        <v>46317.537389317135</v>
       </c>
       <c r="Q105" s="8">
         <v>1</v>
@@ -8181,7 +8181,7 @@
         <v>46315.41700231482</v>
       </c>
       <c r="P106" s="3">
-        <v>46317.53180380787</v>
+        <v>46317.53738854166</v>
       </c>
       <c r="Q106" s="8">
         <v>0</v>
@@ -8258,7 +8258,7 @@
         <v>46315.41678240741</v>
       </c>
       <c r="P107" s="3">
-        <v>46317.53180420139</v>
+        <v>46317.53738892361</v>
       </c>
       <c r="Q107" s="8">
         <v>0</v>
@@ -8330,7 +8330,7 @@
         <v>46315.41725694445</v>
       </c>
       <c r="P108" s="3">
-        <v>46317.53180420139</v>
+        <v>46317.53738892361</v>
       </c>
       <c r="Q108" s="8">
         <v>0</v>
@@ -8407,7 +8407,7 @@
         <v>46315.41703703704</v>
       </c>
       <c r="P109" s="3">
-        <v>46317.531804583334</v>
+        <v>46317.537389317135</v>
       </c>
       <c r="Q109" s="8">
         <v>0</v>
@@ -8484,7 +8484,7 @@
         <v>46315.41681712963</v>
       </c>
       <c r="P110" s="3">
-        <v>46317.531804583334</v>
+        <v>46317.537389317135</v>
       </c>
       <c r="Q110" s="8">
         <v>0</v>
@@ -8561,7 +8561,7 @@
         <v>46315.41729166667</v>
       </c>
       <c r="P111" s="3">
-        <v>46317.531804583334</v>
+        <v>46317.537389317135</v>
       </c>
       <c r="Q111" s="8">
         <v>1</v>
@@ -8633,7 +8633,7 @@
         <v>46315.41729166667</v>
       </c>
       <c r="P112" s="3">
-        <v>46317.53180380787</v>
+        <v>46317.53738854166</v>
       </c>
       <c r="Q112" s="8">
         <v>1</v>
@@ -8705,7 +8705,7 @@
         <v>46315.417071759264</v>
       </c>
       <c r="P113" s="3">
-        <v>46317.53180380787</v>
+        <v>46317.53738854166</v>
       </c>
       <c r="Q113" s="8">
         <v>0</v>
@@ -8777,7 +8777,7 @@
         <v>46315.416851851856</v>
       </c>
       <c r="P114" s="3">
-        <v>46317.53180420139</v>
+        <v>46317.53738892361</v>
       </c>
       <c r="Q114" s="8">
         <v>0</v>
@@ -8849,7 +8849,7 @@
         <v>46315.41732638889</v>
       </c>
       <c r="P115" s="3">
-        <v>46317.53180420139</v>
+        <v>46317.53738892361</v>
       </c>
       <c r="Q115" s="8">
         <v>0</v>
@@ -8921,7 +8921,7 @@
         <v>46315.41710648148</v>
       </c>
       <c r="P116" s="3">
-        <v>46317.531804583334</v>
+        <v>46317.537389317135</v>
       </c>
       <c r="Q116" s="8">
         <v>0</v>
@@ -8988,7 +8988,7 @@
         <v>46315.41688657408</v>
       </c>
       <c r="P117" s="3">
-        <v>46317.53189219907</v>
+        <v>46317.53747668982</v>
       </c>
       <c r="Q117" s="8">
         <v>0</v>

</xml_diff>

<commit_message>
Mobile polish from iPhone review: date field, report-settings popup, camera + gallery buttons, compact project header
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/poc-output/m9-chromium/export-filtered.xlsx
+++ b/poc-output/m9-chromium/export-filtered.xlsx
@@ -293,7 +293,7 @@
         <v>46315.41677083333</v>
       </c>
       <c r="P2" s="3">
-        <v>46317.53738854166</v>
+        <v>46317.6225643287</v>
       </c>
       <c r="Q2" s="8">
         <v>0</v>
@@ -365,7 +365,7 @@
         <v>46315.417245370365</v>
       </c>
       <c r="P3" s="3">
-        <v>46317.53738892361</v>
+        <v>46317.62256469908</v>
       </c>
       <c r="Q3" s="8">
         <v>0</v>
@@ -437,7 +437,7 @@
         <v>46315.417025462964</v>
       </c>
       <c r="P4" s="3">
-        <v>46317.53747668982</v>
+        <v>46317.62265923611</v>
       </c>
       <c r="Q4" s="8">
         <v>0</v>
@@ -509,7 +509,7 @@
         <v>46315.41680555556</v>
       </c>
       <c r="P5" s="3">
-        <v>46317.53738892361</v>
+        <v>46317.62256469908</v>
       </c>
       <c r="Q5" s="8">
         <v>1</v>
@@ -581,7 +581,7 @@
         <v>46315.41728009259</v>
       </c>
       <c r="P6" s="3">
-        <v>46317.53746143519</v>
+        <v>46317.622643229166</v>
       </c>
       <c r="Q6" s="8">
         <v>0</v>
@@ -653,7 +653,7 @@
         <v>46315.41706018518</v>
       </c>
       <c r="P7" s="3">
-        <v>46317.537389317135</v>
+        <v>46317.62256506944</v>
       </c>
       <c r="Q7" s="8">
         <v>0</v>
@@ -720,7 +720,7 @@
         <v>46315.41684027778</v>
       </c>
       <c r="P8" s="3">
-        <v>46317.53738854166</v>
+        <v>46317.6225643287</v>
       </c>
       <c r="Q8" s="8">
         <v>3</v>
@@ -792,7 +792,7 @@
         <v>46315.41731481481</v>
       </c>
       <c r="P9" s="3">
-        <v>46317.53746143519</v>
+        <v>46317.622643229166</v>
       </c>
       <c r="Q9" s="8">
         <v>0</v>
@@ -864,7 +864,7 @@
         <v>46315.4170949074</v>
       </c>
       <c r="P10" s="3">
-        <v>46317.53738892361</v>
+        <v>46317.62256469908</v>
       </c>
       <c r="Q10" s="8">
         <v>0</v>
@@ -936,7 +936,7 @@
         <v>46315.416874999995</v>
       </c>
       <c r="P11" s="3">
-        <v>46317.53738892361</v>
+        <v>46317.62256469908</v>
       </c>
       <c r="Q11" s="8">
         <v>1</v>
@@ -1008,7 +1008,7 @@
         <v>46315.417349537034</v>
       </c>
       <c r="P12" s="3">
-        <v>46317.537389317135</v>
+        <v>46317.62256506944</v>
       </c>
       <c r="Q12" s="8">
         <v>0</v>
@@ -1080,7 +1080,7 @@
         <v>46315.417129629626</v>
       </c>
       <c r="P13" s="3">
-        <v>46317.537389317135</v>
+        <v>46317.62256506944</v>
       </c>
       <c r="Q13" s="8">
         <v>0</v>
@@ -1157,7 +1157,7 @@
         <v>46315.41690972222</v>
       </c>
       <c r="P14" s="3">
-        <v>46317.53738854166</v>
+        <v>46317.6225643287</v>
       </c>
       <c r="Q14" s="8">
         <v>0</v>
@@ -1234,7 +1234,7 @@
         <v>46315.41668981481</v>
       </c>
       <c r="P15" s="3">
-        <v>46317.53738892361</v>
+        <v>46317.62256469908</v>
       </c>
       <c r="Q15" s="8">
         <v>0</v>
@@ -1306,7 +1306,7 @@
         <v>46315.41716435185</v>
       </c>
       <c r="P16" s="3">
-        <v>46317.53738892361</v>
+        <v>46317.62256469908</v>
       </c>
       <c r="Q16" s="8">
         <v>0</v>
@@ -1383,7 +1383,7 @@
         <v>46315.41694444444</v>
       </c>
       <c r="P17" s="3">
-        <v>46317.537389317135</v>
+        <v>46317.62256506944</v>
       </c>
       <c r="Q17" s="8">
         <v>1</v>
@@ -1460,7 +1460,7 @@
         <v>46315.41672453703</v>
       </c>
       <c r="P18" s="3">
-        <v>46317.537389317135</v>
+        <v>46317.62256506944</v>
       </c>
       <c r="Q18" s="8">
         <v>0</v>
@@ -1537,7 +1537,7 @@
         <v>46315.41719907407</v>
       </c>
       <c r="P19" s="3">
-        <v>46317.53747668982</v>
+        <v>46317.62265923611</v>
       </c>
       <c r="Q19" s="8">
         <v>0</v>
@@ -1614,7 +1614,7 @@
         <v>46315.416979166665</v>
       </c>
       <c r="P20" s="3">
-        <v>46317.53738854166</v>
+        <v>46317.6225643287</v>
       </c>
       <c r="Q20" s="8">
         <v>0</v>
@@ -1691,7 +1691,7 @@
         <v>46315.41675925926</v>
       </c>
       <c r="P21" s="3">
-        <v>46317.53738892361</v>
+        <v>46317.62256469908</v>
       </c>
       <c r="Q21" s="8">
         <v>0</v>
@@ -1768,7 +1768,7 @@
         <v>46315.417233796295</v>
       </c>
       <c r="P22" s="3">
-        <v>46317.53747668982</v>
+        <v>46317.62265923611</v>
       </c>
       <c r="Q22" s="8">
         <v>0</v>
@@ -1845,7 +1845,7 @@
         <v>46315.41701388889</v>
       </c>
       <c r="P23" s="3">
-        <v>46317.537389317135</v>
+        <v>46317.62256506944</v>
       </c>
       <c r="Q23" s="8">
         <v>3</v>
@@ -1917,7 +1917,7 @@
         <v>46315.41679398148</v>
       </c>
       <c r="P24" s="3">
-        <v>46317.53746143519</v>
+        <v>46317.622643229166</v>
       </c>
       <c r="Q24" s="8">
         <v>0</v>
@@ -1994,7 +1994,7 @@
         <v>46315.41726851852</v>
       </c>
       <c r="P25" s="3">
-        <v>46317.537389317135</v>
+        <v>46317.62256506944</v>
       </c>
       <c r="Q25" s="8">
         <v>0</v>
@@ -2071,7 +2071,7 @@
         <v>46315.41726851852</v>
       </c>
       <c r="P26" s="3">
-        <v>46317.53747668982</v>
+        <v>46317.62265923611</v>
       </c>
       <c r="Q26" s="8">
         <v>0</v>
@@ -2148,7 +2148,7 @@
         <v>46315.41704861111</v>
       </c>
       <c r="P27" s="3">
-        <v>46317.53738854166</v>
+        <v>46317.6225643287</v>
       </c>
       <c r="Q27" s="8">
         <v>0</v>
@@ -2225,7 +2225,7 @@
         <v>46315.4168287037</v>
       </c>
       <c r="P28" s="3">
-        <v>46317.53746143519</v>
+        <v>46317.622643229166</v>
       </c>
       <c r="Q28" s="8">
         <v>0</v>
@@ -2302,7 +2302,7 @@
         <v>46315.41730324074</v>
       </c>
       <c r="P29" s="3">
-        <v>46317.53738892361</v>
+        <v>46317.62256469908</v>
       </c>
       <c r="Q29" s="8">
         <v>0</v>
@@ -2379,7 +2379,7 @@
         <v>46315.417083333334</v>
       </c>
       <c r="P30" s="3">
-        <v>46317.537389317135</v>
+        <v>46317.62256506944</v>
       </c>
       <c r="Q30" s="8">
         <v>1</v>
@@ -2456,7 +2456,7 @@
         <v>46315.416863425926</v>
       </c>
       <c r="P31" s="3">
-        <v>46317.537389317135</v>
+        <v>46317.62256506944</v>
       </c>
       <c r="Q31" s="8">
         <v>0</v>
@@ -2533,7 +2533,7 @@
         <v>46315.417337962965</v>
       </c>
       <c r="P32" s="3">
-        <v>46317.537389317135</v>
+        <v>46317.62256506944</v>
       </c>
       <c r="Q32" s="8">
         <v>0</v>
@@ -2610,7 +2610,7 @@
         <v>46315.417337962965</v>
       </c>
       <c r="P33" s="3">
-        <v>46317.53738854166</v>
+        <v>46317.6225643287</v>
       </c>
       <c r="Q33" s="8">
         <v>0</v>
@@ -2682,7 +2682,7 @@
         <v>46315.41711805556</v>
       </c>
       <c r="P34" s="3">
-        <v>46317.53738854166</v>
+        <v>46317.6225643287</v>
       </c>
       <c r="Q34" s="8">
         <v>0</v>
@@ -2759,7 +2759,7 @@
         <v>46315.41689814815</v>
       </c>
       <c r="P35" s="3">
-        <v>46317.53738892361</v>
+        <v>46317.62256469908</v>
       </c>
       <c r="Q35" s="8">
         <v>0</v>
@@ -2836,7 +2836,7 @@
         <v>46315.41667824074</v>
       </c>
       <c r="P36" s="3">
-        <v>46317.53738892361</v>
+        <v>46317.62256469908</v>
       </c>
       <c r="Q36" s="8">
         <v>0</v>
@@ -2913,7 +2913,7 @@
         <v>46315.41715277778</v>
       </c>
       <c r="P37" s="3">
-        <v>46317.537389317135</v>
+        <v>46317.62256506944</v>
       </c>
       <c r="Q37" s="8">
         <v>1</v>
@@ -2990,7 +2990,7 @@
         <v>46315.41693287037</v>
       </c>
       <c r="P38" s="3">
-        <v>46317.537389317135</v>
+        <v>46317.62256506944</v>
       </c>
       <c r="Q38" s="8">
         <v>0</v>
@@ -3067,7 +3067,7 @@
         <v>46315.416712962964</v>
       </c>
       <c r="P39" s="3">
-        <v>46317.53738854166</v>
+        <v>46317.6225643287</v>
       </c>
       <c r="Q39" s="8">
         <v>0</v>
@@ -3144,7 +3144,7 @@
         <v>46315.4171875</v>
       </c>
       <c r="P40" s="3">
-        <v>46317.53738892361</v>
+        <v>46317.62256469908</v>
       </c>
       <c r="Q40" s="8">
         <v>3</v>
@@ -3221,7 +3221,7 @@
         <v>46315.416967592595</v>
       </c>
       <c r="P41" s="3">
-        <v>46317.53738892361</v>
+        <v>46317.62256469908</v>
       </c>
       <c r="Q41" s="8">
         <v>0</v>
@@ -3293,7 +3293,7 @@
         <v>46315.41674768519</v>
       </c>
       <c r="P42" s="3">
-        <v>46317.53747668982</v>
+        <v>46317.62265923611</v>
       </c>
       <c r="Q42" s="8">
         <v>0</v>
@@ -3370,7 +3370,7 @@
         <v>46315.417222222226</v>
       </c>
       <c r="P43" s="3">
-        <v>46317.537389317135</v>
+        <v>46317.62256506944</v>
       </c>
       <c r="Q43" s="8">
         <v>1</v>
@@ -3447,7 +3447,7 @@
         <v>46315.41700231482</v>
       </c>
       <c r="P44" s="3">
-        <v>46317.537389317135</v>
+        <v>46317.62256506944</v>
       </c>
       <c r="Q44" s="8">
         <v>0</v>
@@ -3524,7 +3524,7 @@
         <v>46315.41678240741</v>
       </c>
       <c r="P45" s="3">
-        <v>46317.53747668982</v>
+        <v>46317.62265923611</v>
       </c>
       <c r="Q45" s="8">
         <v>0</v>
@@ -3601,7 +3601,7 @@
         <v>46315.41725694445</v>
       </c>
       <c r="P46" s="3">
-        <v>46317.53738892361</v>
+        <v>46317.62256469908</v>
       </c>
       <c r="Q46" s="8">
         <v>0</v>
@@ -3678,7 +3678,7 @@
         <v>46315.41703703704</v>
       </c>
       <c r="P47" s="3">
-        <v>46317.53738892361</v>
+        <v>46317.62256469908</v>
       </c>
       <c r="Q47" s="8">
         <v>0</v>
@@ -3755,7 +3755,7 @@
         <v>46315.41681712963</v>
       </c>
       <c r="P48" s="3">
-        <v>46317.53738892361</v>
+        <v>46317.62256469908</v>
       </c>
       <c r="Q48" s="8">
         <v>0</v>
@@ -3832,7 +3832,7 @@
         <v>46315.41729166667</v>
       </c>
       <c r="P49" s="3">
-        <v>46317.537389317135</v>
+        <v>46317.62256506944</v>
       </c>
       <c r="Q49" s="8">
         <v>1</v>
@@ -3904,7 +3904,7 @@
         <v>46315.417071759264</v>
       </c>
       <c r="P50" s="3">
-        <v>46317.537389317135</v>
+        <v>46317.62256506944</v>
       </c>
       <c r="Q50" s="8">
         <v>0</v>
@@ -3981,7 +3981,7 @@
         <v>46315.416851851856</v>
       </c>
       <c r="P51" s="3">
-        <v>46317.53738854166</v>
+        <v>46317.6225643287</v>
       </c>
       <c r="Q51" s="8">
         <v>0</v>
@@ -4058,7 +4058,7 @@
         <v>46315.41732638889</v>
       </c>
       <c r="P52" s="3">
-        <v>46317.53738892361</v>
+        <v>46317.62256469908</v>
       </c>
       <c r="Q52" s="8">
         <v>0</v>
@@ -4135,7 +4135,7 @@
         <v>46315.41710648148</v>
       </c>
       <c r="P53" s="3">
-        <v>46317.53738892361</v>
+        <v>46317.62256469908</v>
       </c>
       <c r="Q53" s="8">
         <v>0</v>
@@ -4212,7 +4212,7 @@
         <v>46315.41688657408</v>
       </c>
       <c r="P54" s="3">
-        <v>46317.53738892361</v>
+        <v>46317.62256469908</v>
       </c>
       <c r="Q54" s="8">
         <v>0</v>
@@ -4289,7 +4289,7 @@
         <v>46315.41666666667</v>
       </c>
       <c r="P55" s="3">
-        <v>46317.537389317135</v>
+        <v>46317.62256506944</v>
       </c>
       <c r="Q55" s="8">
         <v>3</v>
@@ -4366,7 +4366,7 @@
         <v>46315.4171412037</v>
       </c>
       <c r="P56" s="3">
-        <v>46317.537389317135</v>
+        <v>46317.62256506944</v>
       </c>
       <c r="Q56" s="8">
         <v>0</v>
@@ -4443,7 +4443,7 @@
         <v>46315.416921296295</v>
       </c>
       <c r="P57" s="3">
-        <v>46317.53738854166</v>
+        <v>46317.6225643287</v>
       </c>
       <c r="Q57" s="8">
         <v>0</v>
@@ -4515,7 +4515,7 @@
         <v>46315.41670138889</v>
       </c>
       <c r="P58" s="3">
-        <v>46317.53738892361</v>
+        <v>46317.62256469908</v>
       </c>
       <c r="Q58" s="8">
         <v>0</v>
@@ -4592,7 +4592,7 @@
         <v>46315.417175925926</v>
       </c>
       <c r="P59" s="3">
-        <v>46317.53738892361</v>
+        <v>46317.62256469908</v>
       </c>
       <c r="Q59" s="8">
         <v>0</v>
@@ -4669,7 +4669,7 @@
         <v>46315.41695601852</v>
       </c>
       <c r="P60" s="3">
-        <v>46317.53747668982</v>
+        <v>46317.62265923611</v>
       </c>
       <c r="Q60" s="8">
         <v>0</v>
@@ -4746,7 +4746,7 @@
         <v>46315.41673611111</v>
       </c>
       <c r="P61" s="3">
-        <v>46317.537389317135</v>
+        <v>46317.62256506944</v>
       </c>
       <c r="Q61" s="8">
         <v>1</v>
@@ -4823,7 +4823,7 @@
         <v>46315.41721064815</v>
       </c>
       <c r="P62" s="3">
-        <v>46317.53746143519</v>
+        <v>46317.622643229166</v>
       </c>
       <c r="Q62" s="8">
         <v>0</v>
@@ -4900,7 +4900,7 @@
         <v>46315.41699074074</v>
       </c>
       <c r="P63" s="3">
-        <v>46317.53747668982</v>
+        <v>46317.62265923611</v>
       </c>
       <c r="Q63" s="8">
         <v>0</v>
@@ -4977,7 +4977,7 @@
         <v>46315.41677083333</v>
       </c>
       <c r="P64" s="3">
-        <v>46317.53738892361</v>
+        <v>46317.62256469908</v>
       </c>
       <c r="Q64" s="8">
         <v>0</v>
@@ -5054,7 +5054,7 @@
         <v>46315.417245370365</v>
       </c>
       <c r="P65" s="3">
-        <v>46317.53746143519</v>
+        <v>46317.622643229166</v>
       </c>
       <c r="Q65" s="8">
         <v>0</v>
@@ -5126,7 +5126,7 @@
         <v>46315.417025462964</v>
       </c>
       <c r="P66" s="3">
-        <v>46317.537389317135</v>
+        <v>46317.62256506944</v>
       </c>
       <c r="Q66" s="8">
         <v>0</v>
@@ -5203,7 +5203,7 @@
         <v>46315.41680555556</v>
       </c>
       <c r="P67" s="3">
-        <v>46317.537389317135</v>
+        <v>46317.62256506944</v>
       </c>
       <c r="Q67" s="8">
         <v>1</v>
@@ -5280,7 +5280,7 @@
         <v>46315.41728009259</v>
       </c>
       <c r="P68" s="3">
-        <v>46317.537389317135</v>
+        <v>46317.62256506944</v>
       </c>
       <c r="Q68" s="8">
         <v>0</v>
@@ -5357,7 +5357,7 @@
         <v>46315.41728009259</v>
       </c>
       <c r="P69" s="3">
-        <v>46317.53746143519</v>
+        <v>46317.622643229166</v>
       </c>
       <c r="Q69" s="8">
         <v>0</v>
@@ -5434,7 +5434,7 @@
         <v>46315.41706018518</v>
       </c>
       <c r="P70" s="3">
-        <v>46317.53738854166</v>
+        <v>46317.6225643287</v>
       </c>
       <c r="Q70" s="8">
         <v>0</v>
@@ -5511,7 +5511,7 @@
         <v>46315.41684027778</v>
       </c>
       <c r="P71" s="3">
-        <v>46317.53738892361</v>
+        <v>46317.62256469908</v>
       </c>
       <c r="Q71" s="8">
         <v>3</v>
@@ -5588,7 +5588,7 @@
         <v>46315.41731481481</v>
       </c>
       <c r="P72" s="3">
-        <v>46317.53738892361</v>
+        <v>46317.62256469908</v>
       </c>
       <c r="Q72" s="8">
         <v>0</v>
@@ -5665,7 +5665,7 @@
         <v>46315.4170949074</v>
       </c>
       <c r="P73" s="3">
-        <v>46317.537389317135</v>
+        <v>46317.62256506944</v>
       </c>
       <c r="Q73" s="8">
         <v>0</v>
@@ -5742,7 +5742,7 @@
         <v>46315.416874999995</v>
       </c>
       <c r="P74" s="3">
-        <v>46317.537389317135</v>
+        <v>46317.62256506944</v>
       </c>
       <c r="Q74" s="8">
         <v>1</v>
@@ -5814,7 +5814,7 @@
         <v>46315.417349537034</v>
       </c>
       <c r="P75" s="3">
-        <v>46317.537389317135</v>
+        <v>46317.62256506944</v>
       </c>
       <c r="Q75" s="8">
         <v>0</v>
@@ -5886,7 +5886,7 @@
         <v>46315.417349537034</v>
       </c>
       <c r="P76" s="3">
-        <v>46317.53738854166</v>
+        <v>46317.6225643287</v>
       </c>
       <c r="Q76" s="8">
         <v>0</v>
@@ -5963,7 +5963,7 @@
         <v>46315.417129629626</v>
       </c>
       <c r="P77" s="3">
-        <v>46317.53738892361</v>
+        <v>46317.62256469908</v>
       </c>
       <c r="Q77" s="8">
         <v>0</v>
@@ -6040,7 +6040,7 @@
         <v>46315.41690972222</v>
       </c>
       <c r="P78" s="3">
-        <v>46317.53738892361</v>
+        <v>46317.62256469908</v>
       </c>
       <c r="Q78" s="8">
         <v>0</v>
@@ -6117,7 +6117,7 @@
         <v>46315.41668981481</v>
       </c>
       <c r="P79" s="3">
-        <v>46317.53738892361</v>
+        <v>46317.62256469908</v>
       </c>
       <c r="Q79" s="8">
         <v>0</v>
@@ -6194,7 +6194,7 @@
         <v>46315.41716435185</v>
       </c>
       <c r="P80" s="3">
-        <v>46317.53747668982</v>
+        <v>46317.62265923611</v>
       </c>
       <c r="Q80" s="8">
         <v>0</v>
@@ -6271,7 +6271,7 @@
         <v>46315.41694444444</v>
       </c>
       <c r="P81" s="3">
-        <v>46317.537389317135</v>
+        <v>46317.62256506944</v>
       </c>
       <c r="Q81" s="8">
         <v>1</v>
@@ -6348,7 +6348,7 @@
         <v>46315.41672453703</v>
       </c>
       <c r="P82" s="3">
-        <v>46317.53738854166</v>
+        <v>46317.6225643287</v>
       </c>
       <c r="Q82" s="8">
         <v>0</v>
@@ -6425,7 +6425,7 @@
         <v>46315.41719907407</v>
       </c>
       <c r="P83" s="3">
-        <v>46317.53747668982</v>
+        <v>46317.62265923611</v>
       </c>
       <c r="Q83" s="8">
         <v>0</v>
@@ -6497,7 +6497,7 @@
         <v>46315.416979166665</v>
       </c>
       <c r="P84" s="3">
-        <v>46317.53738892361</v>
+        <v>46317.62256469908</v>
       </c>
       <c r="Q84" s="8">
         <v>0</v>
@@ -6574,7 +6574,7 @@
         <v>46315.41675925926</v>
       </c>
       <c r="P85" s="3">
-        <v>46317.53738892361</v>
+        <v>46317.62256469908</v>
       </c>
       <c r="Q85" s="8">
         <v>0</v>
@@ -6651,7 +6651,7 @@
         <v>46315.417233796295</v>
       </c>
       <c r="P86" s="3">
-        <v>46317.537389317135</v>
+        <v>46317.62256506944</v>
       </c>
       <c r="Q86" s="8">
         <v>0</v>
@@ -6728,7 +6728,7 @@
         <v>46315.41701388889</v>
       </c>
       <c r="P87" s="3">
-        <v>46317.537389317135</v>
+        <v>46317.62256506944</v>
       </c>
       <c r="Q87" s="8">
         <v>3</v>
@@ -6805,7 +6805,7 @@
         <v>46315.41679398148</v>
       </c>
       <c r="P88" s="3">
-        <v>46317.53738854166</v>
+        <v>46317.6225643287</v>
       </c>
       <c r="Q88" s="8">
         <v>0</v>
@@ -6882,7 +6882,7 @@
         <v>46315.41726851852</v>
       </c>
       <c r="P89" s="3">
-        <v>46317.53738892361</v>
+        <v>46317.62256469908</v>
       </c>
       <c r="Q89" s="8">
         <v>0</v>
@@ -6959,7 +6959,7 @@
         <v>46315.41704861111</v>
       </c>
       <c r="P90" s="3">
-        <v>46317.53738892361</v>
+        <v>46317.62256469908</v>
       </c>
       <c r="Q90" s="8">
         <v>0</v>
@@ -7036,7 +7036,7 @@
         <v>46315.4168287037</v>
       </c>
       <c r="P91" s="3">
-        <v>46317.53738892361</v>
+        <v>46317.62256469908</v>
       </c>
       <c r="Q91" s="8">
         <v>0</v>
@@ -7108,7 +7108,7 @@
         <v>46315.41730324074</v>
       </c>
       <c r="P92" s="3">
-        <v>46317.537389317135</v>
+        <v>46317.62256506944</v>
       </c>
       <c r="Q92" s="8">
         <v>0</v>
@@ -7185,7 +7185,7 @@
         <v>46315.417083333334</v>
       </c>
       <c r="P93" s="3">
-        <v>46317.537389317135</v>
+        <v>46317.62256506944</v>
       </c>
       <c r="Q93" s="8">
         <v>1</v>
@@ -7262,7 +7262,7 @@
         <v>46315.416863425926</v>
       </c>
       <c r="P94" s="3">
-        <v>46317.53738854166</v>
+        <v>46317.6225643287</v>
       </c>
       <c r="Q94" s="8">
         <v>0</v>
@@ -7339,7 +7339,7 @@
         <v>46315.417337962965</v>
       </c>
       <c r="P95" s="3">
-        <v>46317.53738892361</v>
+        <v>46317.62256469908</v>
       </c>
       <c r="Q95" s="8">
         <v>0</v>
@@ -7416,7 +7416,7 @@
         <v>46315.41711805556</v>
       </c>
       <c r="P96" s="3">
-        <v>46317.53738892361</v>
+        <v>46317.62256469908</v>
       </c>
       <c r="Q96" s="8">
         <v>0</v>
@@ -7493,7 +7493,7 @@
         <v>46315.41689814815</v>
       </c>
       <c r="P97" s="3">
-        <v>46317.537389317135</v>
+        <v>46317.62256506944</v>
       </c>
       <c r="Q97" s="8">
         <v>0</v>
@@ -7570,7 +7570,7 @@
         <v>46315.41667824074</v>
       </c>
       <c r="P98" s="3">
-        <v>46317.53747668982</v>
+        <v>46317.62265923611</v>
       </c>
       <c r="Q98" s="8">
         <v>0</v>
@@ -7647,7 +7647,7 @@
         <v>46315.41715277778</v>
       </c>
       <c r="P99" s="3">
-        <v>46317.537389317135</v>
+        <v>46317.62256506944</v>
       </c>
       <c r="Q99" s="8">
         <v>1</v>
@@ -7719,7 +7719,7 @@
         <v>46315.41693287037</v>
       </c>
       <c r="P100" s="3">
-        <v>46317.53738854166</v>
+        <v>46317.6225643287</v>
       </c>
       <c r="Q100" s="8">
         <v>0</v>
@@ -7796,7 +7796,7 @@
         <v>46315.416712962964</v>
       </c>
       <c r="P101" s="3">
-        <v>46317.53747668982</v>
+        <v>46317.62265923611</v>
       </c>
       <c r="Q101" s="8">
         <v>0</v>
@@ -7873,7 +7873,7 @@
         <v>46315.4171875</v>
       </c>
       <c r="P102" s="3">
-        <v>46317.53738892361</v>
+        <v>46317.62256469908</v>
       </c>
       <c r="Q102" s="8">
         <v>3</v>
@@ -7950,7 +7950,7 @@
         <v>46315.416967592595</v>
       </c>
       <c r="P103" s="3">
-        <v>46317.537389317135</v>
+        <v>46317.62256506944</v>
       </c>
       <c r="Q103" s="8">
         <v>0</v>
@@ -8027,7 +8027,7 @@
         <v>46315.41674768519</v>
       </c>
       <c r="P104" s="3">
-        <v>46317.537389317135</v>
+        <v>46317.62256506944</v>
       </c>
       <c r="Q104" s="8">
         <v>0</v>
@@ -8104,7 +8104,7 @@
         <v>46315.417222222226</v>
       </c>
       <c r="P105" s="3">
-        <v>46317.537389317135</v>
+        <v>46317.62256506944</v>
       </c>
       <c r="Q105" s="8">
         <v>1</v>
@@ -8181,7 +8181,7 @@
         <v>46315.41700231482</v>
       </c>
       <c r="P106" s="3">
-        <v>46317.53738854166</v>
+        <v>46317.6225643287</v>
       </c>
       <c r="Q106" s="8">
         <v>0</v>
@@ -8258,7 +8258,7 @@
         <v>46315.41678240741</v>
       </c>
       <c r="P107" s="3">
-        <v>46317.53738892361</v>
+        <v>46317.62256469908</v>
       </c>
       <c r="Q107" s="8">
         <v>0</v>
@@ -8330,7 +8330,7 @@
         <v>46315.41725694445</v>
       </c>
       <c r="P108" s="3">
-        <v>46317.53738892361</v>
+        <v>46317.62256469908</v>
       </c>
       <c r="Q108" s="8">
         <v>0</v>
@@ -8407,7 +8407,7 @@
         <v>46315.41703703704</v>
       </c>
       <c r="P109" s="3">
-        <v>46317.537389317135</v>
+        <v>46317.62256506944</v>
       </c>
       <c r="Q109" s="8">
         <v>0</v>
@@ -8484,7 +8484,7 @@
         <v>46315.41681712963</v>
       </c>
       <c r="P110" s="3">
-        <v>46317.537389317135</v>
+        <v>46317.62256506944</v>
       </c>
       <c r="Q110" s="8">
         <v>0</v>
@@ -8561,7 +8561,7 @@
         <v>46315.41729166667</v>
       </c>
       <c r="P111" s="3">
-        <v>46317.537389317135</v>
+        <v>46317.62256506944</v>
       </c>
       <c r="Q111" s="8">
         <v>1</v>
@@ -8633,7 +8633,7 @@
         <v>46315.41729166667</v>
       </c>
       <c r="P112" s="3">
-        <v>46317.53738854166</v>
+        <v>46317.6225643287</v>
       </c>
       <c r="Q112" s="8">
         <v>1</v>
@@ -8705,7 +8705,7 @@
         <v>46315.417071759264</v>
       </c>
       <c r="P113" s="3">
-        <v>46317.53738854166</v>
+        <v>46317.6225643287</v>
       </c>
       <c r="Q113" s="8">
         <v>0</v>
@@ -8777,7 +8777,7 @@
         <v>46315.416851851856</v>
       </c>
       <c r="P114" s="3">
-        <v>46317.53738892361</v>
+        <v>46317.62256469908</v>
       </c>
       <c r="Q114" s="8">
         <v>0</v>
@@ -8849,7 +8849,7 @@
         <v>46315.41732638889</v>
       </c>
       <c r="P115" s="3">
-        <v>46317.53738892361</v>
+        <v>46317.62256469908</v>
       </c>
       <c r="Q115" s="8">
         <v>0</v>
@@ -8921,7 +8921,7 @@
         <v>46315.41710648148</v>
       </c>
       <c r="P116" s="3">
-        <v>46317.537389317135</v>
+        <v>46317.62256506944</v>
       </c>
       <c r="Q116" s="8">
         <v>0</v>
@@ -8988,7 +8988,7 @@
         <v>46315.41688657408</v>
       </c>
       <c r="P117" s="3">
-        <v>46317.53747668982</v>
+        <v>46317.62265923611</v>
       </c>
       <c r="Q117" s="8">
         <v>0</v>

</xml_diff>